<commit_message>
refactor(data): remove native handler version field
</commit_message>
<xml_diff>
--- a/config/data/NativeHandler.xlsx
+++ b/config/data/NativeHandler.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="33">
   <si>
     <t>@table</t>
   </si>
@@ -43,7 +43,7 @@
     <t>@schema</t>
   </si>
   <si>
-    <t>672e41ba07d08321</t>
+    <t>162a5f35ebf31c95</t>
   </si>
   <si>
     <t>#name</t>
@@ -55,9 +55,6 @@
     <t>domain</t>
   </si>
   <si>
-    <t>handler_version</t>
-  </si>
-  <si>
     <t>argument_schema_sha256</t>
   </si>
   <si>
@@ -104,9 +101,6 @@
   </si>
   <si>
     <t>length=1..160</t>
-  </si>
-  <si>
-    <t>length=1..80</t>
   </si>
   <si>
     <t>length=64..64</t>
@@ -125,7 +119,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -133,16 +127,68 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F2937"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2F3A4A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE9EEF5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3D6E8F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDE5EF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8FB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7DB"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -150,12 +196,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -450,216 +529,235 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" style="5" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="22.7109375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" style="5" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" style="5" customWidth="1"/>
+    <col min="8" max="8" width="23.7109375" style="5" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" style="5" customWidth="1"/>
+    <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
-      <c r="A2" t="s">
+    <row r="2" spans="1:10" ht="24" customHeight="1">
+      <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="K2" t="s">
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
         <v>19</v>
       </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="3" spans="1:11">
-      <c r="A3" t="s">
+    <row r="4" spans="1:10">
+      <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" t="s">
-        <v>19</v>
+      <c r="B4" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
-      <c r="A4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" t="s">
-        <v>23</v>
-      </c>
-      <c r="J4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" t="s">
+    <row r="5" spans="1:10">
+      <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
+      <c r="B5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="5" spans="1:11">
-      <c r="A5" t="s">
+    <row r="6" spans="1:10">
+      <c r="A6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" t="s">
-        <v>7</v>
-      </c>
-      <c r="I5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J5" t="s">
-        <v>7</v>
-      </c>
-      <c r="K5" t="s">
-        <v>7</v>
-      </c>
+      <c r="B6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" s="5"/>
     </row>
-    <row r="6" spans="1:11">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" t="s">
+    <row r="7" spans="1:10" ht="42" customHeight="1">
+      <c r="A7" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H6" t="s">
-        <v>33</v>
-      </c>
-      <c r="I6" t="s">
-        <v>32</v>
-      </c>
-      <c r="J6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11">
-      <c r="A7" t="s">
-        <v>34</v>
-      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Value outside range" error="Value must be an integer from 1 to 2147483647." promptTitle="Integer range" prompt="Enter an integer from 1 to 2147483647." sqref="B8:B1007">
+      <formula1>1</formula1>
+      <formula2>2147483647</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Battle, Activity" promptTitle="RuleDomain enum" prompt="Select a value from the dropdown." sqref="D8:D1007">
+      <formula1>"Battle,Activity"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="J8:J1007">
+      <formula1>"true,false"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>